<commit_message>
fix(23127259): finalize confirmed FR14 defect reports (5 bugs)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/23127259/excel/HW06_Test_Cases.xlsx
+++ b/23127259/excel/HW06_Test_Cases.xlsx
@@ -7465,7 +7465,7 @@
         <v>42</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
         <v>46</v>
@@ -7484,7 +7484,7 @@
         <v>120</v>
       </c>
       <c r="C5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" t="n">
         <v>132</v>
@@ -7504,7 +7504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7581,7 +7581,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR02-001.md; FR02 newman Run02</t>
+          <t>23127259/bugs/issues/BUG-FR02-001.md; FR02 newman Run03</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -7618,7 +7618,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR02-002.md</t>
+          <t>23127259/bugs/issues/BUG-FR02-002.md</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR02-003.md</t>
+          <t>23127259/bugs/issues/BUG-FR02-003.md</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -7803,7 +7803,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-001.md; FR14 Run05</t>
+          <t>23127259/bugs/BUG-FR14-001.md; FR14 Run01</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -7840,7 +7840,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-002.md; FR14 Run05</t>
+          <t>23127259/bugs/BUG-FR14-002.md; FR14 Run01</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-003.md; FR14 Run05</t>
+          <t>23127259/bugs/BUG-FR14-003.md; FR14 Run01</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Empty PUT body returns HTTP 500 (robustness)</t>
+          <t>Empty PUT body corrupts existing category name to null</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -7914,12 +7914,49 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-004.md; FR14 Run05</t>
+          <t>23127259/bugs/BUG-FR14-004.md; FR14 Run01</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CONFIRMED (non-normative robustness defect)</t>
+          <t>CONFIRMED (FR-14 corruption is normative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BUG-FR14-005</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>FR14</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PUT/DELETE on already-deleted category returns false-success</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PENDING_GH_ISSUE</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>23127259/bugs/BUG-FR14-005.md; FR14 Run01</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CONFIRMED (FR-14 CRUD integrity)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(23127259): align final reports to 5 FR14 bugs / 6 Human extensions (Run01 canonical)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/23127259/excel/HW06_Test_Cases.xlsx
+++ b/23127259/excel/HW06_Test_Cases.xlsx
@@ -7380,14 +7380,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7398,20 +7399,25 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Raw AI Count</t>
+          <t>Raw AI</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Human Count</t>
+          <t>Usable AI</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Formal Count</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Formal</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Canonical JSON Cases</t>
         </is>
@@ -7427,14 +7433,17 @@
         <v>37</v>
       </c>
       <c r="C2" t="n">
+        <v>35</v>
+      </c>
+      <c r="D2" t="n">
         <v>5</v>
-      </c>
-      <c r="D2" t="n">
-        <v>40</v>
       </c>
       <c r="E2" t="n">
         <v>40</v>
       </c>
+      <c r="F2" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7443,17 +7452,20 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>42</v>
+      </c>
+      <c r="C3" t="n">
         <v>41</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>5</v>
-      </c>
-      <c r="D3" t="n">
-        <v>46</v>
       </c>
       <c r="E3" t="n">
         <v>46</v>
       </c>
+      <c r="F3" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7465,14 +7477,17 @@
         <v>42</v>
       </c>
       <c r="C4" t="n">
+        <v>40</v>
+      </c>
+      <c r="D4" t="n">
         <v>6</v>
-      </c>
-      <c r="D4" t="n">
-        <v>46</v>
       </c>
       <c r="E4" t="n">
         <v>46</v>
       </c>
+      <c r="F4" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7481,15 +7496,18 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C5" t="n">
+        <v>116</v>
+      </c>
+      <c r="D5" t="n">
         <v>16</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>132</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>132</v>
       </c>
     </row>
@@ -7581,7 +7599,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>23127259/bugs/issues/BUG-FR02-001.md; FR02 newman Run03</t>
+          <t>23127259/bugs/BUG-FR02-001.md; FR02 newman Run02</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -7618,7 +7636,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>23127259/bugs/issues/BUG-FR02-002.md</t>
+          <t>23127259/bugs/BUG-FR02-002.md</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -7655,7 +7673,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>23127259/bugs/issues/BUG-FR02-003.md</t>
+          <t>23127259/bugs/BUG-FR02-003.md</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -7867,7 +7885,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Non-existent category update/delete returns 200 with stale payload</t>
+          <t>Non-existent category update/delete returns 200 with false-success</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -7899,7 +7917,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -7909,17 +7927,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PENDING_GH_ISSUE</t>
+          <t>PENDING_GH_ISSUE (GH_AUTH_REQUIRED); body: BUG-FR14-004-issue-body.md</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-004.md; FR14 Run01</t>
+          <t>23127259/bugs/BUG-FR14-004.md; FR14 Run01 (TC-FR14-H05)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CONFIRMED (FR-14 corruption is normative)</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
     </row>
@@ -7941,22 +7959,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PUT/DELETE on already-deleted category returns false-success</t>
+          <t>Already-deleted category PUT/DELETE returns false-success</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PENDING_GH_ISSUE</t>
+          <t>PENDING_GH_ISSUE (GH_AUTH_REQUIRED); body: BUG-FR14-005-issue-body.md</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-005.md; FR14 Run01</t>
+          <t>23127259/bugs/BUG-FR14-005.md; FR14 Run01 (TC-FR14-037/038)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>CONFIRMED (FR-14 CRUD integrity)</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
excel(23127259): align workbook with 4 unique FR14 root causes
- scripts/build_excel_workbook.py: drop BUG-FR14-005 from the Bugs sheet;
  BUG-FR14-003 row now describes the consolidated root cause
  (nonexistent + already-deleted) with TC-FR14-024/025/037/038. BUG-FR02
  titles updated to match the canonical FR02_BUG_CANDIDATES.md titles.
- scripts/automated_final_checks.py: drop FR14-005 from the expected bug
  report set; the workbook now records 10 confirmed bugs (3+3+4).
- Regenerate HW06_Test_Cases.xlsx with 11 rows in Bugs sheet (header + 10
  bugs), 40/46/46 FR02/FR10/FR14 case counts unchanged.

Refs: #34, #36, #37
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/23127259/excel/HW06_Test_Cases.xlsx
+++ b/23127259/excel/HW06_Test_Cases.xlsx
@@ -7522,7 +7522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7589,17 +7589,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sensitive plaintext password leak in /api/users response</t>
+          <t>Plaintext password disclosed in login response JSON</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PENDING_CODEX_VISUAL_AUDIT</t>
+          <t>https://github.com/thangak18/HW06/issues/1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR02-001.md; FR02 newman Run02</t>
+          <t>23127259/bugs/FR02_BUG_CANDIDATES.md; FR02 Run03 (FR02-AI-028)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -7626,22 +7626,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>No rate limit on /api/login allows brute-force attempts</t>
+          <t>Account remains locked beyond documented 30-second lockout duration</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PENDING_CODEX_VISUAL_AUDIT</t>
+          <t>https://github.com/thangak18/HW06/issues/2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR02-002.md</t>
+          <t>23127259/bugs/FR02_BUG_CANDIDATES.md; FR02 Run03 (FR02-AI-021)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>EXPLORATORY</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
     </row>
@@ -7663,22 +7663,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Account lockout counter not persisted across service restart</t>
+          <t>Premature account lockout on valid login at N=2 boundary</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PENDING_CODEX_VISUAL_AUDIT</t>
+          <t>https://github.com/thangak18/HW06/issues/3</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR02-003.md</t>
+          <t>23127259/bugs/FR02_BUG_CANDIDATES.md; FR02 Run03 (FR02-HUM-003)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>EXPLORATORY</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
     </row>
@@ -7700,7 +7700,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Server allows confirmed -&gt; cancelled transition (RBAC bypass for owner)</t>
+          <t>Owner can cancel a confirmed order after it enters shipping</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7737,7 +7737,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Non-existent order status update returns 200 with echoed payload</t>
+          <t>Canceled terminal order can be transitioned to delivered</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Delivered orders can be re-shipped (state-machine integrity)</t>
+          <t>Regular customer can mutate order status through Admin API</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-001.md; FR14 Run01</t>
+          <t>23127259/bugs/BUG-FR14-001.md; FR14 Run01 (TC-FR14-012..014)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-002.md; FR14 Run01</t>
+          <t>23127259/bugs/BUG-FR14-002.md; FR14 Run01 (TC-FR14-016..019)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -7885,7 +7885,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Non-existent category update/delete returns 200 with false-success</t>
+          <t>Non-existent / already-deleted category update/delete returns false success</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -7895,7 +7895,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>23127259/bugs/BUG-FR14-003.md; FR14 Run01</t>
+          <t>23127259/bugs/BUG-FR14-003.md; FR14 Run01 (TC-FR14-024/025/037/038)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -7927,7 +7927,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PENDING_GH_ISSUE (GH_AUTH_REQUIRED); body: BUG-FR14-004-issue-body.md</t>
+          <t>https://github.com/thangak18/HW06/issues/36</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -7936,43 +7936,6 @@
         </is>
       </c>
       <c r="G11" t="inlineStr">
-        <is>
-          <t>CONFIRMED</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>BUG-FR14-005</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>FR14</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Already-deleted category PUT/DELETE returns false-success</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>PENDING_GH_ISSUE (GH_AUTH_REQUIRED); body: BUG-FR14-005-issue-body.md</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>23127259/bugs/BUG-FR14-005.md; FR14 Run01 (TC-FR14-037/038)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
         <is>
           <t>CONFIRMED</t>
         </is>

</xml_diff>

<commit_message>
fix(23127259): finalize HW06 submission artifacts
</commit_message>
<xml_diff>
--- a/23127259/excel/HW06_Test_Cases.xlsx
+++ b/23127259/excel/HW06_Test_Cases.xlsx
@@ -462,7 +462,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Student ID: 23127259</t>
+          <t>Student: Nguyễn Tấn Thắng (MSSV: 23127259)</t>
         </is>
       </c>
     </row>
@@ -483,7 +483,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Visual workbook validation: PENDING_CODEX_VISUAL_AUDIT</t>
+          <t>Visual workbook validation: PASS - All 6 sheets verified complete and compliant</t>
         </is>
       </c>
     </row>

</xml_diff>